<commit_message>
feat: persistent activity logging with Historial dashboard and updated campaign reports
- Added persistent activity storage in db/actividad.json
- Implemented Historial tab with monthly analytics, push grouping, and advisor stats
- Automatic system event logging on snapshot/push
- Mexico City timezone for all timestamps
- Updated graduacion and legion centurion Excel data
</commit_message>
<xml_diff>
--- a/graduacion/graduacion.xlsx
+++ b/graduacion/graduacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/diego/Desktop/panel de campañas/graduacion/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D09B9A5-3944-9742-AB06-23F4420B783A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B89D1F8C-3D05-3E41-B3AF-72D8F884D3B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="500" windowWidth="24460" windowHeight="16360" xr2:uid="{C790F585-E5F8-714F-8D00-C112DB38F0A1}"/>
   </bookViews>
@@ -390,47 +390,7 @@
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="59">
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
+  <dxfs count="42">
     <dxf>
       <font>
         <b/>
@@ -496,8 +456,17 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FFFF0000"/>
-      </font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF00B0F0"/>
+        <name val="Cambria"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -517,10 +486,15 @@
       <font>
         <b/>
         <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
+        <color rgb="FF0070C0"/>
+        <name val="Cambria"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -538,10 +512,220 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="10"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <color indexed="16"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="31"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="hair">
+          <color indexed="64"/>
+        </left>
+        <right style="hair">
+          <color indexed="64"/>
+        </right>
+        <top style="hair">
+          <color indexed="64"/>
+        </top>
+        <bottom style="hair">
+          <color indexed="64"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <border>
         <left style="hair">
           <color indexed="64"/>
@@ -574,132 +758,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B0F0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF0070C0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <border>
         <left style="thin">
           <color theme="0" tint="-0.14996795556505021"/>
@@ -716,430 +774,6 @@
       </border>
     </dxf>
     <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="16"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="31"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B0F0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF0070C0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFC00000"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B0F0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF0070C0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF00B0F0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF0070C0"/>
-        <name val="Cambria"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="10"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FFFF0000"/>
-      </font>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <color indexed="16"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="31"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="hair">
-          <color indexed="64"/>
-        </left>
-        <right style="hair">
-          <color indexed="64"/>
-        </right>
-        <top style="hair">
-          <color indexed="64"/>
-        </top>
-        <bottom style="hair">
-          <color indexed="64"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border>
-        <left style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </left>
-        <right style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </right>
-        <top style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </top>
-        <bottom style="thin">
-          <color theme="0" tint="-0.14996795556505021"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1628,32 +1262,32 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8C84689-1448-8442-B1F2-C8CC1CDB3E89}" name="Tabla1" displayName="Tabla1" ref="A3:W15" totalsRowShown="0" headerRowDxfId="58">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{C8C84689-1448-8442-B1F2-C8CC1CDB3E89}" name="Tabla1" displayName="Tabla1" ref="A3:W15" totalsRowShown="0" headerRowDxfId="41">
   <autoFilter ref="A3:W15" xr:uid="{C8C84689-1448-8442-B1F2-C8CC1CDB3E89}"/>
   <tableColumns count="23">
-    <tableColumn id="1" xr3:uid="{3B622300-6924-DB4F-A62F-2EEC39FAB0A2}" name="DIR / ZONA" dataDxfId="57"/>
-    <tableColumn id="2" xr3:uid="{56109AD6-9361-EA49-82CB-5F16E0E8FEF7}" name="OFICINA" dataDxfId="56"/>
-    <tableColumn id="3" xr3:uid="{AB1E1DBC-B048-A740-9A78-5965EB9EC44F}" name="GERENCIA / SP" dataDxfId="55"/>
-    <tableColumn id="4" xr3:uid="{61CAAE43-B726-6C46-97AC-90058F4DA6D1}" name="MAT" dataDxfId="54"/>
-    <tableColumn id="5" xr3:uid="{E8AA5DF5-9B6D-2543-9325-7C035D241238}" name="SUC" dataDxfId="53"/>
-    <tableColumn id="6" xr3:uid="{295631B1-0185-9B4D-8500-6B9AA08F63F2}" name="PROMOTOR / PARTNER" dataDxfId="52"/>
-    <tableColumn id="7" xr3:uid="{4B47B735-008D-2449-B456-D2DD3B472696}" name="ASESOR" dataDxfId="51"/>
-    <tableColumn id="8" xr3:uid="{975EC707-F2EE-5144-BEFE-BA96A47202F3}" name="NOMBRE" dataDxfId="50"/>
-    <tableColumn id="9" xr3:uid="{027BA34A-24D8-E94B-83B2-B0C1B6025207}" name="MES" dataDxfId="49" dataCellStyle="Millares"/>
-    <tableColumn id="10" xr3:uid="{646ECA88-7396-D040-B5DF-0AAEB243F28F}" name="F. CONEXIÓN" dataDxfId="48" dataCellStyle="Millares"/>
-    <tableColumn id="11" xr3:uid="{26CD5808-6FE4-1F4D-BE8F-7814A14EB008}" name="F. CONCURSO" dataDxfId="47" dataCellStyle="Millares"/>
-    <tableColumn id="12" xr3:uid="{4B28D83F-5D6D-624E-BB91-9704EE1A3E14}" name="LÍMITE P/  LOGRO DE META" dataDxfId="46" dataCellStyle="Millares"/>
-    <tableColumn id="13" xr3:uid="{E489BE13-FD5F-904D-8881-224954582674}" name="CUADERNO DE CONCURSO" dataDxfId="45" dataCellStyle="Millares"/>
-    <tableColumn id="14" xr3:uid="{26915D16-D4BC-B145-BE2F-527AE56B2BAB}" name="GRUPO" dataDxfId="44"/>
-    <tableColumn id="15" xr3:uid="{A89792EE-9143-B14C-9C0C-81844C60721D}" name="TOTAL" dataDxfId="43"/>
-    <tableColumn id="16" xr3:uid="{14F06EE7-B141-B346-AB39-618B1114E96F}" name="CANCEL." dataDxfId="42"/>
-    <tableColumn id="17" xr3:uid="{9B9D77BF-8869-CA44-BCEA-33C8D4FA1307}" name="EN VIGOR" dataDxfId="41"/>
-    <tableColumn id="18" xr3:uid="{2060FD50-AB1E-C245-B146-DB9618552765}" name="PROMEDIO" dataDxfId="40"/>
-    <tableColumn id="19" xr3:uid="{F956BCDA-7715-ED46-9C68-AA2CA74FB455}" name="VIDA" dataDxfId="39"/>
-    <tableColumn id="20" xr3:uid="{F8F35AF9-120D-5944-B380-9F31E59F8709}" name="GMM" dataDxfId="38"/>
-    <tableColumn id="21" xr3:uid="{E6C3EA59-5FA1-3446-9DEF-1B9EE5CF332D}" name="TOTAL2" dataDxfId="37"/>
-    <tableColumn id="22" xr3:uid="{75E46555-9E6E-E349-A48E-06957BB9C039}" name="ESTATUS" dataDxfId="36"/>
-    <tableColumn id="23" xr3:uid="{24832D48-18B2-2F4B-A6BA-E52011154826}" name="OBSERVACIÓN" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{3B622300-6924-DB4F-A62F-2EEC39FAB0A2}" name="DIR / ZONA" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{56109AD6-9361-EA49-82CB-5F16E0E8FEF7}" name="OFICINA" dataDxfId="39"/>
+    <tableColumn id="3" xr3:uid="{AB1E1DBC-B048-A740-9A78-5965EB9EC44F}" name="GERENCIA / SP" dataDxfId="38"/>
+    <tableColumn id="4" xr3:uid="{61CAAE43-B726-6C46-97AC-90058F4DA6D1}" name="MAT" dataDxfId="37"/>
+    <tableColumn id="5" xr3:uid="{E8AA5DF5-9B6D-2543-9325-7C035D241238}" name="SUC" dataDxfId="36"/>
+    <tableColumn id="6" xr3:uid="{295631B1-0185-9B4D-8500-6B9AA08F63F2}" name="PROMOTOR / PARTNER" dataDxfId="35"/>
+    <tableColumn id="7" xr3:uid="{4B47B735-008D-2449-B456-D2DD3B472696}" name="ASESOR" dataDxfId="34"/>
+    <tableColumn id="8" xr3:uid="{975EC707-F2EE-5144-BEFE-BA96A47202F3}" name="NOMBRE" dataDxfId="33"/>
+    <tableColumn id="9" xr3:uid="{027BA34A-24D8-E94B-83B2-B0C1B6025207}" name="MES" dataDxfId="32" dataCellStyle="Millares"/>
+    <tableColumn id="10" xr3:uid="{646ECA88-7396-D040-B5DF-0AAEB243F28F}" name="F. CONEXIÓN" dataDxfId="31" dataCellStyle="Millares"/>
+    <tableColumn id="11" xr3:uid="{26CD5808-6FE4-1F4D-BE8F-7814A14EB008}" name="F. CONCURSO" dataDxfId="30" dataCellStyle="Millares"/>
+    <tableColumn id="12" xr3:uid="{4B28D83F-5D6D-624E-BB91-9704EE1A3E14}" name="LÍMITE P/  LOGRO DE META" dataDxfId="29" dataCellStyle="Millares"/>
+    <tableColumn id="13" xr3:uid="{E489BE13-FD5F-904D-8881-224954582674}" name="CUADERNO DE CONCURSO" dataDxfId="28" dataCellStyle="Millares"/>
+    <tableColumn id="14" xr3:uid="{26915D16-D4BC-B145-BE2F-527AE56B2BAB}" name="GRUPO" dataDxfId="27"/>
+    <tableColumn id="15" xr3:uid="{A89792EE-9143-B14C-9C0C-81844C60721D}" name="TOTAL" dataDxfId="26"/>
+    <tableColumn id="16" xr3:uid="{14F06EE7-B141-B346-AB39-618B1114E96F}" name="CANCEL." dataDxfId="25"/>
+    <tableColumn id="17" xr3:uid="{9B9D77BF-8869-CA44-BCEA-33C8D4FA1307}" name="EN VIGOR" dataDxfId="24"/>
+    <tableColumn id="18" xr3:uid="{2060FD50-AB1E-C245-B146-DB9618552765}" name="PROMEDIO" dataDxfId="23"/>
+    <tableColumn id="19" xr3:uid="{F956BCDA-7715-ED46-9C68-AA2CA74FB455}" name="VIDA" dataDxfId="22"/>
+    <tableColumn id="20" xr3:uid="{F8F35AF9-120D-5944-B380-9F31E59F8709}" name="GMM" dataDxfId="21"/>
+    <tableColumn id="21" xr3:uid="{E6C3EA59-5FA1-3446-9DEF-1B9EE5CF332D}" name="TOTAL2" dataDxfId="20"/>
+    <tableColumn id="22" xr3:uid="{75E46555-9E6E-E349-A48E-06957BB9C039}" name="ESTATUS" dataDxfId="19"/>
+    <tableColumn id="23" xr3:uid="{24832D48-18B2-2F4B-A6BA-E52011154826}" name="OBSERVACIÓN" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2840,90 +2474,57 @@
       <c r="W15" s="29"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="V5:V14">
-    <cfRule type="cellIs" dxfId="22" priority="20" operator="equal">
-      <formula>"Cumplio Meta"</formula>
+  <conditionalFormatting sqref="A5:W14">
+    <cfRule type="expression" dxfId="17" priority="5">
+      <formula>$B5&lt;&gt;""</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="21" operator="equal">
-      <formula>"VM"</formula>
+    <cfRule type="expression" dxfId="16" priority="12">
+      <formula>$B5&lt;&gt;""</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="15" priority="22">
+      <formula>$B5&lt;&gt;""</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5:R14 N5:N14">
-    <cfRule type="expression" dxfId="20" priority="23">
+    <cfRule type="expression" dxfId="14" priority="23">
       <formula>AND($B5&lt;&gt;"",$O5&lt;&gt;"2",,$O5&lt;&gt;"3")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5:Q9">
-    <cfRule type="expression" dxfId="19" priority="19">
+    <cfRule type="expression" dxfId="13" priority="18">
+      <formula>AND($B5&lt;&gt;"",Q5&lt;36)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="19">
       <formula>"y($B18&lt;&gt;"",r18&lt;36)"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q5:Q9">
-    <cfRule type="expression" dxfId="18" priority="18">
+  <conditionalFormatting sqref="Q5:Q14">
+    <cfRule type="expression" dxfId="11" priority="2">
       <formula>AND($B5&lt;&gt;"",Q5&lt;36)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U5:U9">
-    <cfRule type="expression" dxfId="17" priority="17">
-      <formula>AND($B5&lt;&gt;"",U5&lt;95000)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:W14">
-    <cfRule type="expression" dxfId="16" priority="22">
-      <formula>$B5&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:W14">
-    <cfRule type="expression" dxfId="15" priority="12">
-      <formula>$B5&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q5:Q14">
-    <cfRule type="expression" dxfId="14" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>AND($B5&lt;&gt;"",Q5&lt;36)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="R5:R14">
-    <cfRule type="expression" dxfId="13" priority="15">
+    <cfRule type="expression" dxfId="9" priority="8">
+      <formula>AND($J5&gt;=13,$S5&lt;1,$B5&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="15">
       <formula>AND($J5&gt;=13,$S5&lt;1,$B5&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U5:U14">
-    <cfRule type="expression" dxfId="12" priority="16">
+    <cfRule type="expression" dxfId="7" priority="9">
+      <formula>AND($B5&lt;&gt;"",U5&lt;95000)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="16">
       <formula>AND($B5&lt;&gt;"",U5&lt;95000)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V5:V14">
-    <cfRule type="cellIs" dxfId="11" priority="13" operator="equal">
-      <formula>"Cumplio Meta"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="14" operator="equal">
-      <formula>"VM"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W5:W14">
-    <cfRule type="containsText" dxfId="9" priority="10" operator="containsText" text="No cumple">
-      <formula>NOT(ISERROR(SEARCH("No cumple",W5)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:W14">
-    <cfRule type="expression" dxfId="8" priority="5">
-      <formula>$B5&lt;&gt;""</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q5:Q14">
-    <cfRule type="expression" dxfId="7" priority="4">
-      <formula>AND($B5&lt;&gt;"",Q5&lt;36)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R5:R14">
-    <cfRule type="expression" dxfId="6" priority="8">
-      <formula>AND($J5&gt;=13,$S5&lt;1,$B5&lt;&gt;"")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U5:U14">
-    <cfRule type="expression" dxfId="5" priority="9">
-      <formula>AND($B5&lt;&gt;"",U5&lt;95000)</formula>
+  <conditionalFormatting sqref="U10:U14">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>AND($B10&lt;&gt;"",U10&lt;95000)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="V5:V14">
@@ -2933,23 +2534,20 @@
     <cfRule type="cellIs" dxfId="3" priority="7" operator="equal">
       <formula>"VM"</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="13" operator="equal">
+      <formula>"Cumplio Meta"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="14" operator="equal">
+      <formula>"VM"</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W5:W14">
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="No cumple">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="No cumple">
       <formula>NOT(ISERROR(SEARCH("No cumple",W5)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q10:Q14">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>AND($B10&lt;&gt;"",Q10&lt;36)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U10:U14">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>AND($B10&lt;&gt;"",U10&lt;95000)</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>